<commit_message>
v0.2 - Support multiple Excel files
</commit_message>
<xml_diff>
--- a/templates/report_template.xlsx
+++ b/templates/report_template.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/64bab628b403b612/Belgeler/GitHub/ExcelReporter/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="8_{3E3ED728-13CE-4E35-ACF9-2EC2185FA195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0CED2CC-F917-4A9F-8CD5-D3A192400B67}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="8_{3E3ED728-13CE-4E35-ACF9-2EC2185FA195}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{96222AFC-D6B8-4F13-8E8A-50BDB013F631}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5DB07A39-A750-404B-A053-5DA16FF01EC0}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -113,6 +113,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>